<commit_message>
#3 Client and eSpark BOM update acc to current Schematic.
</commit_message>
<xml_diff>
--- a/Design-Files/FMM-v1.0/BOM/Client_BOM.xlsx
+++ b/Design-Files/FMM-v1.0/BOM/Client_BOM.xlsx
@@ -5,7 +5,7 @@
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="153222"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Iftikhar Ahmed\OneDrive\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\eSpark-Consultants\johncox-fmmdesign\Design-Files\FMM-v1.0\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="618" uniqueCount="391">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="620" uniqueCount="394">
   <si>
     <t>#</t>
   </si>
@@ -45,9 +45,6 @@
     <t>Ferrite Bead</t>
   </si>
   <si>
-    <t>Fuse Holder</t>
-  </si>
-  <si>
     <t>Connector</t>
   </si>
   <si>
@@ -165,9 +162,6 @@
     <t>FB1, FB2, FB3, FB4, FB5</t>
   </si>
   <si>
-    <t>J1</t>
-  </si>
-  <si>
     <t>J2</t>
   </si>
   <si>
@@ -405,9 +399,6 @@
     <t>DIODE ZENER 3.3V 200MW SOD323F</t>
   </si>
   <si>
-    <t>TVS DIODE 33VWM 53.3VC SMA</t>
-  </si>
-  <si>
     <t>DIODE SCHOTTKY 20V 500MA SOD123</t>
   </si>
   <si>
@@ -426,9 +417,6 @@
     <t>FERRITE BEAD 1K OHM 0805 1LN</t>
   </si>
   <si>
-    <t>FUSE HOLDER BLADE 80V PCB</t>
-  </si>
-  <si>
     <t>1x6P SH 1 1mm 6 SMD,P=1mm Wire To Board / Wire To Wire Connector ROHS</t>
   </si>
   <si>
@@ -621,9 +609,6 @@
     <t>SOD323F</t>
   </si>
   <si>
-    <t>SMA</t>
-  </si>
-  <si>
     <t>SOD-123</t>
   </si>
   <si>
@@ -642,9 +627,6 @@
     <t>Ind-0805</t>
   </si>
   <si>
-    <t>178.6165.0002</t>
-  </si>
-  <si>
     <t>Voltlink Target</t>
   </si>
   <si>
@@ -780,9 +762,6 @@
     <t>MM3Z3V3B</t>
   </si>
   <si>
-    <t>SMAJ33AQ-13-F</t>
-  </si>
-  <si>
     <t>MBR0520LT1G</t>
   </si>
   <si>
@@ -978,9 +957,6 @@
     <t>TDK</t>
   </si>
   <si>
-    <t>Littelfuse Wickmann</t>
-  </si>
-  <si>
     <t>BOOMELE</t>
   </si>
   <si>
@@ -1192,6 +1168,39 @@
   </si>
   <si>
     <t>KHB65-37(11)-28-A/3</t>
+  </si>
+  <si>
+    <t>TVS DIODE 30VWM 48.4VC SMC</t>
+  </si>
+  <si>
+    <t>SMC</t>
+  </si>
+  <si>
+    <t>3.0SMCJ30AQ-13</t>
+  </si>
+  <si>
+    <t>16V 1A 100A 1.8A 1206 Resettable Fuses ROHS</t>
+  </si>
+  <si>
+    <t>Fuse 1206 (3216 Metric)</t>
+  </si>
+  <si>
+    <t>BSMD1206-100-16V</t>
+  </si>
+  <si>
+    <t>BHFUSE</t>
+  </si>
+  <si>
+    <t>Fuse</t>
+  </si>
+  <si>
+    <t>F1</t>
+  </si>
+  <si>
+    <t>ECU Connector</t>
+  </si>
+  <si>
+    <t>DJ7391-1.5/2.8-11 automotive male 39 pin pcb connector ecu connector</t>
   </si>
 </sst>
 </file>
@@ -1246,17 +1255,20 @@
       <sz val="10"/>
       <color theme="0"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="10"/>
       <color theme="1"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="9"/>
       <color theme="1"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="6">
@@ -1525,9 +1537,6 @@
     <xf numFmtId="0" fontId="5" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1561,6 +1570,9 @@
     </xf>
     <xf numFmtId="0" fontId="8" fillId="5" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1862,6 +1874,9 @@
     <col min="9" max="9" width="6.140625" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="8.7109375" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="8.5703125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="25.28515625" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="8.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -1873,9 +1888,9 @@
       <c r="F1" s="2"/>
       <c r="G1" s="2"/>
       <c r="H1" s="2"/>
-      <c r="I1" s="14"/>
-      <c r="J1" s="14"/>
-      <c r="K1" s="14"/>
+      <c r="I1" s="26"/>
+      <c r="J1" s="26"/>
+      <c r="K1" s="26"/>
     </row>
     <row r="2" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1"/>
@@ -1886,28 +1901,28 @@
         <v>1</v>
       </c>
       <c r="D2" s="5" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E2" s="6" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="F2" s="5" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
       <c r="G2" s="6" t="s">
-        <v>233</v>
+        <v>227</v>
       </c>
       <c r="H2" s="5" t="s">
-        <v>306</v>
+        <v>299</v>
       </c>
       <c r="I2" s="6" t="s">
-        <v>387</v>
+        <v>379</v>
       </c>
       <c r="J2" s="5" t="s">
-        <v>374</v>
+        <v>366</v>
       </c>
       <c r="K2" s="5" t="s">
-        <v>388</v>
+        <v>380</v>
       </c>
     </row>
     <row r="3" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -1920,22 +1935,22 @@
         <v>2</v>
       </c>
       <c r="D3" s="7" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E3" s="8" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="F3" s="7" t="s">
-        <v>192</v>
+        <v>188</v>
       </c>
       <c r="G3" s="8" t="s">
-        <v>234</v>
+        <v>228</v>
       </c>
       <c r="H3" s="7" t="s">
-        <v>307</v>
+        <v>300</v>
       </c>
       <c r="I3" s="8" t="s">
-        <v>330</v>
+        <v>322</v>
       </c>
       <c r="J3" s="7">
         <v>9</v>
@@ -1952,22 +1967,22 @@
         <v>2</v>
       </c>
       <c r="D4" s="9" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="E4" s="10" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="F4" s="9" t="s">
-        <v>192</v>
+        <v>188</v>
       </c>
       <c r="G4" s="10" t="s">
-        <v>235</v>
+        <v>229</v>
       </c>
       <c r="H4" s="9" t="s">
-        <v>307</v>
+        <v>300</v>
       </c>
       <c r="I4" s="10" t="s">
-        <v>331</v>
+        <v>323</v>
       </c>
       <c r="J4" s="9">
         <v>31</v>
@@ -1984,22 +1999,22 @@
         <v>2</v>
       </c>
       <c r="D5" s="7" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E5" s="8" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="F5" s="7" t="s">
-        <v>193</v>
+        <v>189</v>
       </c>
       <c r="G5" s="8" t="s">
-        <v>193</v>
+        <v>189</v>
       </c>
       <c r="H5" s="7" t="s">
-        <v>308</v>
+        <v>301</v>
       </c>
       <c r="I5" s="8" t="s">
-        <v>332</v>
+        <v>324</v>
       </c>
       <c r="J5" s="7">
         <v>2</v>
@@ -2016,22 +2031,22 @@
         <v>2</v>
       </c>
       <c r="D6" s="9" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E6" s="10" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="F6" s="9" t="s">
-        <v>194</v>
+        <v>190</v>
       </c>
       <c r="G6" s="10" t="s">
-        <v>194</v>
+        <v>190</v>
       </c>
       <c r="H6" s="9" t="s">
-        <v>308</v>
+        <v>301</v>
       </c>
       <c r="I6" s="10" t="s">
-        <v>333</v>
+        <v>325</v>
       </c>
       <c r="J6" s="9">
         <v>2</v>
@@ -2048,22 +2063,22 @@
         <v>2</v>
       </c>
       <c r="D7" s="7" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E7" s="8" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="F7" s="7" t="s">
-        <v>195</v>
+        <v>191</v>
       </c>
       <c r="G7" s="8" t="s">
-        <v>236</v>
+        <v>230</v>
       </c>
       <c r="H7" s="7" t="s">
-        <v>309</v>
+        <v>302</v>
       </c>
       <c r="I7" s="8" t="s">
-        <v>334</v>
+        <v>326</v>
       </c>
       <c r="J7" s="7">
         <v>2</v>
@@ -2080,22 +2095,22 @@
         <v>2</v>
       </c>
       <c r="D8" s="9" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="E8" s="10" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="F8" s="9" t="s">
-        <v>195</v>
+        <v>191</v>
       </c>
       <c r="G8" s="10" t="s">
-        <v>237</v>
+        <v>231</v>
       </c>
       <c r="H8" s="9" t="s">
-        <v>309</v>
+        <v>302</v>
       </c>
       <c r="I8" s="10" t="s">
-        <v>335</v>
+        <v>327</v>
       </c>
       <c r="J8" s="9">
         <v>1</v>
@@ -2112,22 +2127,22 @@
         <v>2</v>
       </c>
       <c r="D9" s="7" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E9" s="8" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="F9" s="7" t="s">
-        <v>195</v>
+        <v>191</v>
       </c>
       <c r="G9" s="8" t="s">
-        <v>238</v>
+        <v>232</v>
       </c>
       <c r="H9" s="7" t="s">
-        <v>309</v>
+        <v>302</v>
       </c>
       <c r="I9" s="8" t="s">
-        <v>336</v>
+        <v>328</v>
       </c>
       <c r="J9" s="7">
         <v>1</v>
@@ -2144,22 +2159,22 @@
         <v>2</v>
       </c>
       <c r="D10" s="9" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E10" s="10" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="F10" s="9" t="s">
-        <v>192</v>
+        <v>188</v>
       </c>
       <c r="G10" s="10" t="s">
-        <v>239</v>
+        <v>233</v>
       </c>
       <c r="H10" s="9" t="s">
-        <v>310</v>
+        <v>303</v>
       </c>
       <c r="I10" s="10" t="s">
-        <v>337</v>
+        <v>329</v>
       </c>
       <c r="J10" s="9">
         <v>1</v>
@@ -2176,22 +2191,22 @@
         <v>2</v>
       </c>
       <c r="D11" s="7" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E11" s="8" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="F11" s="7" t="s">
-        <v>192</v>
+        <v>188</v>
       </c>
       <c r="G11" s="8" t="s">
-        <v>240</v>
+        <v>234</v>
       </c>
       <c r="H11" s="7" t="s">
-        <v>310</v>
+        <v>303</v>
       </c>
       <c r="I11" s="8" t="s">
-        <v>338</v>
+        <v>330</v>
       </c>
       <c r="J11" s="7">
         <v>1</v>
@@ -2208,22 +2223,22 @@
         <v>2</v>
       </c>
       <c r="D12" s="9" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="E12" s="10" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="F12" s="9" t="s">
-        <v>195</v>
+        <v>191</v>
       </c>
       <c r="G12" s="10" t="s">
-        <v>241</v>
+        <v>235</v>
       </c>
       <c r="H12" s="9" t="s">
-        <v>307</v>
+        <v>300</v>
       </c>
       <c r="I12" s="10" t="s">
-        <v>339</v>
+        <v>331</v>
       </c>
       <c r="J12" s="9">
         <v>3</v>
@@ -2240,22 +2255,22 @@
         <v>2</v>
       </c>
       <c r="D13" s="7" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="E13" s="8" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="F13" s="7" t="s">
-        <v>196</v>
+        <v>192</v>
       </c>
       <c r="G13" s="8" t="s">
-        <v>242</v>
+        <v>236</v>
       </c>
       <c r="H13" s="7" t="s">
-        <v>310</v>
+        <v>303</v>
       </c>
       <c r="I13" s="8" t="s">
-        <v>340</v>
+        <v>332</v>
       </c>
       <c r="J13" s="7">
         <v>2</v>
@@ -2272,22 +2287,22 @@
         <v>2</v>
       </c>
       <c r="D14" s="9" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="E14" s="10" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="F14" s="9" t="s">
-        <v>192</v>
+        <v>188</v>
       </c>
       <c r="G14" s="10" t="s">
-        <v>243</v>
+        <v>237</v>
       </c>
       <c r="H14" s="9" t="s">
-        <v>309</v>
+        <v>302</v>
       </c>
       <c r="I14" s="10" t="s">
-        <v>330</v>
+        <v>322</v>
       </c>
       <c r="J14" s="9">
         <v>1</v>
@@ -2304,22 +2319,22 @@
         <v>2</v>
       </c>
       <c r="D15" s="7" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="E15" s="8" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="F15" s="7" t="s">
-        <v>192</v>
+        <v>188</v>
       </c>
       <c r="G15" s="8" t="s">
-        <v>244</v>
+        <v>238</v>
       </c>
       <c r="H15" s="7" t="s">
-        <v>309</v>
+        <v>302</v>
       </c>
       <c r="I15" s="8" t="s">
-        <v>332</v>
+        <v>324</v>
       </c>
       <c r="J15" s="7">
         <v>7</v>
@@ -2336,22 +2351,22 @@
         <v>2</v>
       </c>
       <c r="D16" s="9" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E16" s="10" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="F16" s="9" t="s">
-        <v>192</v>
-      </c>
-      <c r="G16" s="22" t="s">
-        <v>385</v>
-      </c>
-      <c r="H16" s="21" t="s">
-        <v>310</v>
+        <v>188</v>
+      </c>
+      <c r="G16" s="21" t="s">
+        <v>377</v>
+      </c>
+      <c r="H16" s="20" t="s">
+        <v>303</v>
       </c>
       <c r="I16" s="10" t="s">
-        <v>341</v>
+        <v>333</v>
       </c>
       <c r="J16" s="9">
         <v>1</v>
@@ -2368,22 +2383,22 @@
         <v>2</v>
       </c>
       <c r="D17" s="7" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E17" s="8" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="F17" s="7" t="s">
-        <v>195</v>
+        <v>191</v>
       </c>
       <c r="G17" s="8" t="s">
-        <v>245</v>
+        <v>239</v>
       </c>
       <c r="H17" s="7" t="s">
-        <v>318</v>
+        <v>311</v>
       </c>
       <c r="I17" s="8" t="s">
-        <v>342</v>
+        <v>334</v>
       </c>
       <c r="J17" s="7">
         <v>2</v>
@@ -2400,22 +2415,22 @@
         <v>2</v>
       </c>
       <c r="D18" s="9" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="E18" s="10" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="F18" s="9" t="s">
-        <v>195</v>
+        <v>191</v>
       </c>
       <c r="G18" s="10" t="s">
-        <v>246</v>
+        <v>240</v>
       </c>
       <c r="H18" s="9" t="s">
-        <v>309</v>
+        <v>302</v>
       </c>
       <c r="I18" s="10" t="s">
-        <v>343</v>
+        <v>335</v>
       </c>
       <c r="J18" s="9">
         <v>1</v>
@@ -2432,22 +2447,22 @@
         <v>2</v>
       </c>
       <c r="D19" s="7" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="E19" s="8" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="F19" s="7" t="s">
-        <v>192</v>
+        <v>188</v>
       </c>
       <c r="G19" s="8" t="s">
-        <v>247</v>
+        <v>241</v>
       </c>
       <c r="H19" s="7" t="s">
-        <v>309</v>
+        <v>302</v>
       </c>
       <c r="I19" s="8" t="s">
-        <v>335</v>
+        <v>327</v>
       </c>
       <c r="J19" s="7">
         <v>12</v>
@@ -2464,22 +2479,22 @@
         <v>2</v>
       </c>
       <c r="D20" s="9" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="E20" s="10" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="F20" s="9" t="s">
-        <v>192</v>
+        <v>188</v>
       </c>
       <c r="G20" s="10" t="s">
-        <v>248</v>
+        <v>242</v>
       </c>
       <c r="H20" s="9" t="s">
-        <v>309</v>
+        <v>302</v>
       </c>
       <c r="I20" s="10" t="s">
-        <v>331</v>
+        <v>323</v>
       </c>
       <c r="J20" s="9">
         <v>4</v>
@@ -2496,22 +2511,22 @@
         <v>2</v>
       </c>
       <c r="D21" s="7" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="E21" s="8" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="F21" s="7" t="s">
-        <v>192</v>
+        <v>188</v>
       </c>
       <c r="G21" s="8" t="s">
-        <v>249</v>
+        <v>243</v>
       </c>
       <c r="H21" s="7" t="s">
-        <v>309</v>
+        <v>302</v>
       </c>
       <c r="I21" s="8" t="s">
-        <v>344</v>
+        <v>336</v>
       </c>
       <c r="J21" s="7">
         <v>4</v>
@@ -2528,22 +2543,22 @@
         <v>3</v>
       </c>
       <c r="D22" s="9" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="E22" s="10" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="F22" s="9" t="s">
-        <v>197</v>
+        <v>193</v>
       </c>
       <c r="G22" s="10" t="s">
-        <v>250</v>
+        <v>244</v>
       </c>
       <c r="H22" s="9" t="s">
-        <v>311</v>
+        <v>304</v>
       </c>
       <c r="I22" s="10" t="s">
-        <v>376</v>
+        <v>368</v>
       </c>
       <c r="J22" s="9">
         <v>1</v>
@@ -2560,22 +2575,22 @@
         <v>3</v>
       </c>
       <c r="D23" s="7" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="E23" s="8" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="F23" s="7" t="s">
-        <v>198</v>
+        <v>194</v>
       </c>
       <c r="G23" s="8" t="s">
-        <v>251</v>
+        <v>245</v>
       </c>
       <c r="H23" s="7" t="s">
-        <v>312</v>
+        <v>305</v>
       </c>
       <c r="I23" s="10" t="s">
-        <v>376</v>
+        <v>368</v>
       </c>
       <c r="J23" s="7">
         <v>1</v>
@@ -2592,22 +2607,22 @@
         <v>3</v>
       </c>
       <c r="D24" s="9" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="E24" s="10" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="F24" s="9" t="s">
-        <v>199</v>
+        <v>195</v>
       </c>
       <c r="G24" s="10" t="s">
-        <v>252</v>
+        <v>246</v>
       </c>
       <c r="H24" s="9" t="s">
-        <v>313</v>
+        <v>306</v>
       </c>
       <c r="I24" s="10" t="s">
-        <v>376</v>
+        <v>368</v>
       </c>
       <c r="J24" s="9">
         <v>1</v>
@@ -2624,22 +2639,22 @@
         <v>3</v>
       </c>
       <c r="D25" s="7" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="E25" s="8" t="s">
-        <v>128</v>
+        <v>383</v>
       </c>
       <c r="F25" s="7" t="s">
-        <v>200</v>
+        <v>384</v>
       </c>
       <c r="G25" s="8" t="s">
-        <v>253</v>
+        <v>385</v>
       </c>
       <c r="H25" s="7" t="s">
-        <v>312</v>
-      </c>
-      <c r="I25" s="10" t="s">
-        <v>376</v>
+        <v>305</v>
+      </c>
+      <c r="I25" s="8" t="s">
+        <v>368</v>
       </c>
       <c r="J25" s="7">
         <v>1</v>
@@ -2656,22 +2671,22 @@
         <v>3</v>
       </c>
       <c r="D26" s="9" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="E26" s="10" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="F26" s="9" t="s">
-        <v>201</v>
+        <v>196</v>
       </c>
       <c r="G26" s="10" t="s">
-        <v>254</v>
+        <v>247</v>
       </c>
       <c r="H26" s="9" t="s">
-        <v>314</v>
+        <v>307</v>
       </c>
       <c r="I26" s="10" t="s">
-        <v>376</v>
+        <v>368</v>
       </c>
       <c r="J26" s="9">
         <v>2</v>
@@ -2688,22 +2703,22 @@
         <v>3</v>
       </c>
       <c r="D27" s="7" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E27" s="8" t="s">
-        <v>130</v>
+        <v>127</v>
       </c>
       <c r="F27" s="7" t="s">
-        <v>202</v>
+        <v>197</v>
       </c>
       <c r="G27" s="8" t="s">
-        <v>255</v>
+        <v>248</v>
       </c>
       <c r="H27" s="7" t="s">
-        <v>315</v>
+        <v>308</v>
       </c>
       <c r="I27" s="10" t="s">
-        <v>376</v>
+        <v>368</v>
       </c>
       <c r="J27" s="7">
         <v>1</v>
@@ -2720,22 +2735,22 @@
         <v>4</v>
       </c>
       <c r="D28" s="9" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="E28" s="10" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="F28" s="9" t="s">
-        <v>203</v>
+        <v>198</v>
       </c>
       <c r="G28" s="10" t="s">
-        <v>256</v>
+        <v>249</v>
       </c>
       <c r="H28" s="9" t="s">
-        <v>316</v>
+        <v>309</v>
       </c>
       <c r="I28" s="10" t="s">
-        <v>376</v>
+        <v>368</v>
       </c>
       <c r="J28" s="9">
         <v>3</v>
@@ -2752,22 +2767,22 @@
         <v>5</v>
       </c>
       <c r="D29" s="7" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="E29" s="8" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
       <c r="F29" s="7" t="s">
-        <v>204</v>
+        <v>199</v>
       </c>
       <c r="G29" s="8" t="s">
-        <v>257</v>
+        <v>250</v>
       </c>
       <c r="H29" s="7" t="s">
-        <v>317</v>
+        <v>310</v>
       </c>
       <c r="I29" s="10" t="s">
-        <v>376</v>
+        <v>368</v>
       </c>
       <c r="J29" s="7">
         <v>1</v>
@@ -2784,91 +2799,91 @@
         <v>6</v>
       </c>
       <c r="D30" s="9" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="E30" s="10" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="F30" s="9" t="s">
-        <v>205</v>
-      </c>
-      <c r="G30" s="19" t="s">
-        <v>345</v>
-      </c>
-      <c r="H30" s="18" t="s">
-        <v>386</v>
+        <v>200</v>
+      </c>
+      <c r="G30" s="18" t="s">
+        <v>337</v>
+      </c>
+      <c r="H30" s="17" t="s">
+        <v>378</v>
       </c>
       <c r="I30" s="10" t="s">
-        <v>376</v>
+        <v>368</v>
       </c>
       <c r="J30" s="9">
         <v>4</v>
       </c>
       <c r="K30" s="9"/>
     </row>
-    <row r="31" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A31" s="1"/>
       <c r="B31" s="11">
-        <f>ROW(B31) - ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>29</v>
       </c>
       <c r="C31" s="12" t="s">
-        <v>7</v>
+        <v>390</v>
       </c>
       <c r="D31" s="7" t="s">
-        <v>47</v>
+        <v>391</v>
       </c>
       <c r="E31" s="8" t="s">
-        <v>134</v>
+        <v>386</v>
       </c>
       <c r="F31" s="7" t="s">
-        <v>206</v>
+        <v>387</v>
       </c>
       <c r="G31" s="8" t="s">
-        <v>258</v>
+        <v>388</v>
       </c>
       <c r="H31" s="7" t="s">
-        <v>318</v>
-      </c>
-      <c r="I31" s="10" t="s">
-        <v>376</v>
+        <v>389</v>
+      </c>
+      <c r="I31" s="8" t="s">
+        <v>368</v>
       </c>
       <c r="J31" s="7">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="K31" s="7"/>
     </row>
     <row r="32" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A32" s="1"/>
       <c r="B32" s="11">
-        <f t="shared" si="0"/>
+        <f>ROW(B32) - ROW($B$2)</f>
         <v>30</v>
       </c>
-      <c r="C32" s="13" t="s">
-        <v>8</v>
-      </c>
-      <c r="D32" s="9" t="s">
-        <v>48</v>
-      </c>
-      <c r="E32" s="10" t="s">
-        <v>135</v>
-      </c>
-      <c r="F32" s="9" t="s">
-        <v>207</v>
-      </c>
-      <c r="G32" s="10" t="s">
-        <v>207</v>
-      </c>
-      <c r="H32" s="9" t="s">
-        <v>319</v>
+      <c r="C32" s="12" t="s">
+        <v>7</v>
+      </c>
+      <c r="D32" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="E32" s="8" t="s">
+        <v>131</v>
+      </c>
+      <c r="F32" s="7" t="s">
+        <v>201</v>
+      </c>
+      <c r="G32" s="8" t="s">
+        <v>251</v>
+      </c>
+      <c r="H32" s="7" t="s">
+        <v>311</v>
       </c>
       <c r="I32" s="10" t="s">
-        <v>376</v>
-      </c>
-      <c r="J32" s="9">
-        <v>1</v>
-      </c>
-      <c r="K32" s="9"/>
+        <v>368</v>
+      </c>
+      <c r="J32" s="7">
+        <v>5</v>
+      </c>
+      <c r="K32" s="7"/>
     </row>
     <row r="33" spans="1:11" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A33" s="1"/>
@@ -2877,49 +2892,53 @@
         <v>31</v>
       </c>
       <c r="C33" s="12" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D33" s="7" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="E33" s="8" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="F33" s="7" t="s">
-        <v>208</v>
+        <v>202</v>
       </c>
       <c r="G33" s="8" t="s">
-        <v>259</v>
+        <v>252</v>
       </c>
       <c r="H33" s="7" t="s">
-        <v>320</v>
+        <v>312</v>
       </c>
       <c r="I33" s="10" t="s">
-        <v>376</v>
+        <v>368</v>
       </c>
       <c r="J33" s="7">
         <v>1</v>
       </c>
       <c r="K33" s="7"/>
     </row>
-    <row r="34" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A34" s="1"/>
       <c r="B34" s="11">
         <f t="shared" si="0"/>
         <v>32</v>
       </c>
-      <c r="C34" s="13"/>
+      <c r="C34" s="13" t="s">
+        <v>392</v>
+      </c>
       <c r="D34" s="9" t="s">
-        <v>50</v>
-      </c>
-      <c r="E34" s="10"/>
+        <v>48</v>
+      </c>
+      <c r="E34" s="10" t="s">
+        <v>393</v>
+      </c>
       <c r="F34" s="9" t="s">
-        <v>209</v>
+        <v>203</v>
       </c>
       <c r="G34" s="10"/>
       <c r="H34" s="9"/>
       <c r="I34" s="10" t="s">
-        <v>376</v>
+        <v>368</v>
       </c>
       <c r="J34" s="9">
         <v>1</v>
@@ -2933,25 +2952,25 @@
         <v>33</v>
       </c>
       <c r="C35" s="12" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D35" s="7" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="E35" s="8" t="s">
-        <v>137</v>
+        <v>133</v>
       </c>
       <c r="F35" s="7" t="s">
-        <v>210</v>
+        <v>204</v>
       </c>
       <c r="G35" s="8" t="s">
-        <v>210</v>
+        <v>204</v>
       </c>
       <c r="H35" s="7" t="s">
-        <v>317</v>
+        <v>310</v>
       </c>
       <c r="I35" s="8" t="s">
-        <v>346</v>
+        <v>338</v>
       </c>
       <c r="J35" s="7">
         <v>1</v>
@@ -2965,25 +2984,25 @@
         <v>34</v>
       </c>
       <c r="C36" s="13" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D36" s="9" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="E36" s="10" t="s">
-        <v>138</v>
+        <v>134</v>
       </c>
       <c r="F36" s="9" t="s">
-        <v>211</v>
+        <v>205</v>
       </c>
       <c r="G36" s="10" t="s">
-        <v>211</v>
+        <v>205</v>
       </c>
       <c r="H36" s="9" t="s">
-        <v>318</v>
+        <v>311</v>
       </c>
       <c r="I36" s="10" t="s">
-        <v>347</v>
+        <v>339</v>
       </c>
       <c r="J36" s="9">
         <v>1</v>
@@ -2997,22 +3016,22 @@
         <v>35</v>
       </c>
       <c r="C37" s="12" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D37" s="7" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="E37" s="8" t="s">
-        <v>139</v>
+        <v>135</v>
       </c>
       <c r="F37" s="7" t="s">
-        <v>212</v>
+        <v>206</v>
       </c>
       <c r="G37" s="8" t="s">
-        <v>212</v>
+        <v>206</v>
       </c>
       <c r="H37" s="7" t="s">
-        <v>318</v>
+        <v>311</v>
       </c>
       <c r="I37" s="8"/>
       <c r="J37" s="7">
@@ -3027,22 +3046,22 @@
         <v>36</v>
       </c>
       <c r="C38" s="13" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D38" s="9" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="E38" s="10" t="s">
-        <v>140</v>
+        <v>136</v>
       </c>
       <c r="F38" s="9" t="s">
-        <v>213</v>
+        <v>207</v>
       </c>
       <c r="G38" s="10" t="s">
-        <v>260</v>
+        <v>253</v>
       </c>
       <c r="H38" s="9" t="s">
-        <v>321</v>
+        <v>313</v>
       </c>
       <c r="I38" s="10"/>
       <c r="J38" s="9">
@@ -3057,22 +3076,22 @@
         <v>37</v>
       </c>
       <c r="C39" s="12" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D39" s="7" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="E39" s="8" t="s">
-        <v>141</v>
+        <v>137</v>
       </c>
       <c r="F39" s="7" t="s">
-        <v>213</v>
+        <v>207</v>
       </c>
       <c r="G39" s="8" t="s">
-        <v>261</v>
+        <v>254</v>
       </c>
       <c r="H39" s="7" t="s">
-        <v>321</v>
+        <v>313</v>
       </c>
       <c r="I39" s="8"/>
       <c r="J39" s="7">
@@ -3087,22 +3106,22 @@
         <v>38</v>
       </c>
       <c r="C40" s="13" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D40" s="9" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="E40" s="10" t="s">
-        <v>142</v>
+        <v>138</v>
       </c>
       <c r="F40" s="9" t="s">
-        <v>213</v>
+        <v>207</v>
       </c>
       <c r="G40" s="10" t="s">
-        <v>262</v>
+        <v>255</v>
       </c>
       <c r="H40" s="9" t="s">
-        <v>321</v>
+        <v>313</v>
       </c>
       <c r="I40" s="10"/>
       <c r="J40" s="9">
@@ -3117,22 +3136,22 @@
         <v>39</v>
       </c>
       <c r="C41" s="12" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D41" s="7" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="E41" s="8" t="s">
-        <v>143</v>
+        <v>139</v>
       </c>
       <c r="F41" s="7" t="s">
-        <v>213</v>
+        <v>207</v>
       </c>
       <c r="G41" s="8" t="s">
-        <v>263</v>
+        <v>256</v>
       </c>
       <c r="H41" s="7" t="s">
-        <v>321</v>
+        <v>313</v>
       </c>
       <c r="I41" s="8"/>
       <c r="J41" s="7">
@@ -3147,22 +3166,22 @@
         <v>40</v>
       </c>
       <c r="C42" s="13" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D42" s="9" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="E42" s="10" t="s">
-        <v>144</v>
+        <v>140</v>
       </c>
       <c r="F42" s="9" t="s">
-        <v>214</v>
+        <v>208</v>
       </c>
       <c r="G42" s="10" t="s">
-        <v>264</v>
+        <v>257</v>
       </c>
       <c r="H42" s="9" t="s">
-        <v>322</v>
+        <v>314</v>
       </c>
       <c r="I42" s="10"/>
       <c r="J42" s="9">
@@ -3177,22 +3196,22 @@
         <v>41</v>
       </c>
       <c r="C43" s="13" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D43" s="7" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="E43" s="8" t="s">
-        <v>145</v>
+        <v>141</v>
       </c>
       <c r="F43" s="7" t="s">
-        <v>215</v>
+        <v>209</v>
       </c>
       <c r="G43" s="8" t="s">
-        <v>265</v>
+        <v>258</v>
       </c>
       <c r="H43" s="7" t="s">
-        <v>322</v>
+        <v>314</v>
       </c>
       <c r="I43" s="8"/>
       <c r="J43" s="7">
@@ -3207,22 +3226,22 @@
         <v>42</v>
       </c>
       <c r="C44" s="13" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D44" s="9" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="E44" s="10" t="s">
-        <v>146</v>
+        <v>142</v>
       </c>
       <c r="F44" s="9" t="s">
-        <v>204</v>
+        <v>199</v>
       </c>
       <c r="G44" s="10" t="s">
-        <v>266</v>
+        <v>259</v>
       </c>
       <c r="H44" s="9" t="s">
-        <v>323</v>
+        <v>315</v>
       </c>
       <c r="I44" s="10"/>
       <c r="J44" s="9">
@@ -3237,25 +3256,25 @@
         <v>43</v>
       </c>
       <c r="C45" s="12" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D45" s="7" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="E45" s="8" t="s">
-        <v>147</v>
+        <v>143</v>
       </c>
       <c r="F45" s="7" t="s">
-        <v>216</v>
+        <v>210</v>
       </c>
       <c r="G45" s="8" t="s">
-        <v>267</v>
+        <v>260</v>
       </c>
       <c r="H45" s="7" t="s">
-        <v>309</v>
+        <v>302</v>
       </c>
       <c r="I45" s="8" t="s">
-        <v>348</v>
+        <v>340</v>
       </c>
       <c r="J45" s="7">
         <v>1</v>
@@ -3269,25 +3288,25 @@
         <v>44</v>
       </c>
       <c r="C46" s="13" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D46" s="9" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="E46" s="10" t="s">
-        <v>148</v>
+        <v>144</v>
       </c>
       <c r="F46" s="9" t="s">
-        <v>217</v>
+        <v>211</v>
       </c>
       <c r="G46" s="10" t="s">
-        <v>268</v>
+        <v>261</v>
       </c>
       <c r="H46" s="9" t="s">
-        <v>309</v>
+        <v>302</v>
       </c>
       <c r="I46" s="10" t="s">
-        <v>349</v>
+        <v>341</v>
       </c>
       <c r="J46" s="9">
         <v>1</v>
@@ -3301,25 +3320,25 @@
         <v>45</v>
       </c>
       <c r="C47" s="12" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D47" s="7" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="E47" s="8" t="s">
-        <v>149</v>
+        <v>145</v>
       </c>
       <c r="F47" s="7" t="s">
-        <v>216</v>
+        <v>210</v>
       </c>
       <c r="G47" s="8" t="s">
-        <v>269</v>
+        <v>262</v>
       </c>
       <c r="H47" s="7" t="s">
-        <v>309</v>
+        <v>302</v>
       </c>
       <c r="I47" s="8" t="s">
-        <v>350</v>
+        <v>342</v>
       </c>
       <c r="J47" s="7">
         <v>1</v>
@@ -3333,25 +3352,25 @@
         <v>46</v>
       </c>
       <c r="C48" s="13" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D48" s="9" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="E48" s="10" t="s">
-        <v>150</v>
+        <v>146</v>
       </c>
       <c r="F48" s="9" t="s">
-        <v>217</v>
+        <v>211</v>
       </c>
       <c r="G48" s="10" t="s">
-        <v>270</v>
+        <v>263</v>
       </c>
       <c r="H48" s="9" t="s">
-        <v>309</v>
+        <v>302</v>
       </c>
       <c r="I48" s="10" t="s">
-        <v>351</v>
+        <v>343</v>
       </c>
       <c r="J48" s="9">
         <v>1</v>
@@ -3365,25 +3384,25 @@
         <v>47</v>
       </c>
       <c r="C49" s="12" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D49" s="7" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="E49" s="8" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="F49" s="7" t="s">
-        <v>218</v>
+        <v>212</v>
       </c>
       <c r="G49" s="8" t="s">
-        <v>271</v>
+        <v>264</v>
       </c>
       <c r="H49" s="7" t="s">
-        <v>317</v>
+        <v>310</v>
       </c>
       <c r="I49" s="8" t="s">
-        <v>352</v>
+        <v>344</v>
       </c>
       <c r="J49" s="7">
         <v>1</v>
@@ -3397,25 +3416,25 @@
         <v>48</v>
       </c>
       <c r="C50" s="13" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D50" s="9" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="E50" s="10" t="s">
-        <v>152</v>
+        <v>148</v>
       </c>
       <c r="F50" s="9" t="s">
-        <v>216</v>
+        <v>210</v>
       </c>
       <c r="G50" s="10" t="s">
-        <v>272</v>
+        <v>265</v>
       </c>
       <c r="H50" s="9" t="s">
-        <v>309</v>
+        <v>302</v>
       </c>
       <c r="I50" s="10" t="s">
-        <v>353</v>
+        <v>345</v>
       </c>
       <c r="J50" s="9">
         <v>1</v>
@@ -3429,25 +3448,25 @@
         <v>49</v>
       </c>
       <c r="C51" s="12" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D51" s="7" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="E51" s="8" t="s">
-        <v>153</v>
+        <v>149</v>
       </c>
       <c r="F51" s="7" t="s">
-        <v>216</v>
+        <v>210</v>
       </c>
       <c r="G51" s="8" t="s">
-        <v>273</v>
+        <v>266</v>
       </c>
       <c r="H51" s="7" t="s">
-        <v>309</v>
+        <v>302</v>
       </c>
       <c r="I51" s="8" t="s">
-        <v>354</v>
+        <v>346</v>
       </c>
       <c r="J51" s="7">
         <v>1</v>
@@ -3461,25 +3480,25 @@
         <v>50</v>
       </c>
       <c r="C52" s="13" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D52" s="9" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="E52" s="10" t="s">
-        <v>154</v>
+        <v>150</v>
       </c>
       <c r="F52" s="9" t="s">
-        <v>216</v>
+        <v>210</v>
       </c>
       <c r="G52" s="10" t="s">
-        <v>274</v>
+        <v>267</v>
       </c>
       <c r="H52" s="9" t="s">
-        <v>309</v>
+        <v>302</v>
       </c>
       <c r="I52" s="10" t="s">
-        <v>355</v>
+        <v>347</v>
       </c>
       <c r="J52" s="9">
         <v>1</v>
@@ -3493,25 +3512,25 @@
         <v>51</v>
       </c>
       <c r="C53" s="12" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D53" s="7" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="E53" s="8" t="s">
-        <v>155</v>
+        <v>151</v>
       </c>
       <c r="F53" s="7" t="s">
-        <v>216</v>
+        <v>210</v>
       </c>
       <c r="G53" s="8" t="s">
-        <v>275</v>
+        <v>268</v>
       </c>
       <c r="H53" s="7" t="s">
-        <v>309</v>
+        <v>302</v>
       </c>
       <c r="I53" s="8" t="s">
-        <v>356</v>
+        <v>348</v>
       </c>
       <c r="J53" s="7">
         <v>1</v>
@@ -3525,25 +3544,25 @@
         <v>52</v>
       </c>
       <c r="C54" s="12" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D54" s="9" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="E54" s="10" t="s">
-        <v>156</v>
+        <v>152</v>
       </c>
       <c r="F54" s="9" t="s">
-        <v>216</v>
+        <v>210</v>
       </c>
       <c r="G54" s="10" t="s">
-        <v>276</v>
+        <v>269</v>
       </c>
       <c r="H54" s="9" t="s">
-        <v>309</v>
+        <v>302</v>
       </c>
       <c r="I54" s="10" t="s">
-        <v>357</v>
+        <v>349</v>
       </c>
       <c r="J54" s="9">
         <v>1</v>
@@ -3557,25 +3576,25 @@
         <v>53</v>
       </c>
       <c r="C55" s="12" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D55" s="7" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="E55" s="8" t="s">
-        <v>157</v>
+        <v>153</v>
       </c>
       <c r="F55" s="7" t="s">
-        <v>216</v>
+        <v>210</v>
       </c>
       <c r="G55" s="8" t="s">
-        <v>277</v>
+        <v>270</v>
       </c>
       <c r="H55" s="7" t="s">
-        <v>309</v>
+        <v>302</v>
       </c>
       <c r="I55" s="8" t="s">
-        <v>358</v>
+        <v>350</v>
       </c>
       <c r="J55" s="7">
         <v>5</v>
@@ -3589,25 +3608,25 @@
         <v>54</v>
       </c>
       <c r="C56" s="12" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D56" s="9" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="E56" s="10" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
       <c r="F56" s="9" t="s">
-        <v>216</v>
+        <v>210</v>
       </c>
       <c r="G56" s="10" t="s">
-        <v>278</v>
+        <v>271</v>
       </c>
       <c r="H56" s="9" t="s">
-        <v>309</v>
+        <v>302</v>
       </c>
       <c r="I56" s="10" t="s">
-        <v>359</v>
+        <v>351</v>
       </c>
       <c r="J56" s="9">
         <v>1</v>
@@ -3621,25 +3640,25 @@
         <v>55</v>
       </c>
       <c r="C57" s="12" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D57" s="7" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="E57" s="8" t="s">
-        <v>159</v>
+        <v>155</v>
       </c>
       <c r="F57" s="7" t="s">
-        <v>216</v>
+        <v>210</v>
       </c>
       <c r="G57" s="8" t="s">
-        <v>279</v>
+        <v>272</v>
       </c>
       <c r="H57" s="7" t="s">
-        <v>309</v>
+        <v>302</v>
       </c>
       <c r="I57" s="8" t="s">
-        <v>360</v>
+        <v>352</v>
       </c>
       <c r="J57" s="7">
         <v>1</v>
@@ -3653,25 +3672,25 @@
         <v>56</v>
       </c>
       <c r="C58" s="12" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D58" s="9" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="E58" s="10" t="s">
-        <v>160</v>
+        <v>156</v>
       </c>
       <c r="F58" s="9" t="s">
-        <v>216</v>
+        <v>210</v>
       </c>
       <c r="G58" s="10" t="s">
-        <v>280</v>
+        <v>273</v>
       </c>
       <c r="H58" s="9" t="s">
-        <v>309</v>
+        <v>302</v>
       </c>
       <c r="I58" s="10" t="s">
-        <v>361</v>
+        <v>353</v>
       </c>
       <c r="J58" s="9">
         <v>1</v>
@@ -3685,25 +3704,25 @@
         <v>57</v>
       </c>
       <c r="C59" s="12" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D59" s="7" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="E59" s="8" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
       <c r="F59" s="7" t="s">
-        <v>216</v>
-      </c>
-      <c r="G59" s="22" t="s">
-        <v>389</v>
+        <v>210</v>
+      </c>
+      <c r="G59" s="21" t="s">
+        <v>381</v>
       </c>
       <c r="H59" s="9" t="s">
-        <v>309</v>
+        <v>302</v>
       </c>
       <c r="I59" s="8" t="s">
-        <v>362</v>
+        <v>354</v>
       </c>
       <c r="J59" s="7">
         <v>1</v>
@@ -3717,25 +3736,25 @@
         <v>58</v>
       </c>
       <c r="C60" s="13" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D60" s="9" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="E60" s="10" t="s">
-        <v>162</v>
+        <v>158</v>
       </c>
       <c r="F60" s="9" t="s">
-        <v>217</v>
+        <v>211</v>
       </c>
       <c r="G60" s="10" t="s">
-        <v>281</v>
+        <v>274</v>
       </c>
       <c r="H60" s="9" t="s">
-        <v>309</v>
+        <v>302</v>
       </c>
       <c r="I60" s="10" t="s">
-        <v>363</v>
+        <v>355</v>
       </c>
       <c r="J60" s="9">
         <v>1</v>
@@ -3749,25 +3768,25 @@
         <v>59</v>
       </c>
       <c r="C61" s="12" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D61" s="7" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="E61" s="8" t="s">
-        <v>163</v>
+        <v>159</v>
       </c>
       <c r="F61" s="7" t="s">
-        <v>216</v>
+        <v>210</v>
       </c>
       <c r="G61" s="8" t="s">
-        <v>282</v>
+        <v>275</v>
       </c>
       <c r="H61" s="7" t="s">
-        <v>309</v>
+        <v>302</v>
       </c>
       <c r="I61" s="8" t="s">
-        <v>356</v>
+        <v>348</v>
       </c>
       <c r="J61" s="7">
         <v>6</v>
@@ -3781,25 +3800,25 @@
         <v>60</v>
       </c>
       <c r="C62" s="13" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D62" s="9" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="E62" s="10" t="s">
-        <v>164</v>
+        <v>160</v>
       </c>
       <c r="F62" s="9" t="s">
-        <v>217</v>
+        <v>211</v>
       </c>
       <c r="G62" s="10" t="s">
-        <v>283</v>
+        <v>276</v>
       </c>
       <c r="H62" s="9" t="s">
-        <v>309</v>
+        <v>302</v>
       </c>
       <c r="I62" s="10" t="s">
-        <v>364</v>
+        <v>356</v>
       </c>
       <c r="J62" s="9">
         <v>2</v>
@@ -3813,25 +3832,25 @@
         <v>61</v>
       </c>
       <c r="C63" s="12" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D63" s="7" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="E63" s="8" t="s">
-        <v>165</v>
+        <v>161</v>
       </c>
       <c r="F63" s="7" t="s">
-        <v>217</v>
+        <v>211</v>
       </c>
       <c r="G63" s="8" t="s">
-        <v>284</v>
+        <v>277</v>
       </c>
       <c r="H63" s="7" t="s">
-        <v>309</v>
+        <v>302</v>
       </c>
       <c r="I63" s="8" t="s">
-        <v>365</v>
+        <v>357</v>
       </c>
       <c r="J63" s="7">
         <v>1</v>
@@ -3845,25 +3864,25 @@
         <v>62</v>
       </c>
       <c r="C64" s="13" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D64" s="9" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="E64" s="10" t="s">
-        <v>166</v>
+        <v>162</v>
       </c>
       <c r="F64" s="9" t="s">
-        <v>217</v>
+        <v>211</v>
       </c>
       <c r="G64" s="10" t="s">
-        <v>285</v>
+        <v>278</v>
       </c>
       <c r="H64" s="9" t="s">
-        <v>309</v>
+        <v>302</v>
       </c>
       <c r="I64" s="10" t="s">
-        <v>366</v>
+        <v>358</v>
       </c>
       <c r="J64" s="9">
         <v>1</v>
@@ -3877,25 +3896,25 @@
         <v>63</v>
       </c>
       <c r="C65" s="13" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D65" s="7" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="E65" s="8" t="s">
-        <v>167</v>
+        <v>163</v>
       </c>
       <c r="F65" s="7" t="s">
-        <v>217</v>
+        <v>211</v>
       </c>
       <c r="G65" s="8" t="s">
-        <v>286</v>
+        <v>279</v>
       </c>
       <c r="H65" s="7" t="s">
-        <v>309</v>
+        <v>302</v>
       </c>
       <c r="I65" s="8" t="s">
-        <v>361</v>
+        <v>353</v>
       </c>
       <c r="J65" s="7">
         <v>1</v>
@@ -3909,25 +3928,25 @@
         <v>64</v>
       </c>
       <c r="C66" s="13" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D66" s="9" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="E66" s="10" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="F66" s="9" t="s">
-        <v>216</v>
+        <v>210</v>
       </c>
       <c r="G66" s="10" t="s">
-        <v>287</v>
+        <v>280</v>
       </c>
       <c r="H66" s="9" t="s">
-        <v>309</v>
+        <v>302</v>
       </c>
       <c r="I66" s="10" t="s">
-        <v>367</v>
+        <v>359</v>
       </c>
       <c r="J66" s="9">
         <v>2</v>
@@ -3941,25 +3960,25 @@
         <v>65</v>
       </c>
       <c r="C67" s="13" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D67" s="7" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="E67" s="8" t="s">
-        <v>169</v>
+        <v>165</v>
       </c>
       <c r="F67" s="7" t="s">
-        <v>217</v>
+        <v>211</v>
       </c>
       <c r="G67" s="8" t="s">
-        <v>288</v>
+        <v>281</v>
       </c>
       <c r="H67" s="7" t="s">
-        <v>309</v>
+        <v>302</v>
       </c>
       <c r="I67" s="8" t="s">
-        <v>368</v>
+        <v>360</v>
       </c>
       <c r="J67" s="7">
         <v>1</v>
@@ -3973,25 +3992,25 @@
         <v>66</v>
       </c>
       <c r="C68" s="13" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D68" s="9" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="E68" s="10" t="s">
-        <v>170</v>
+        <v>166</v>
       </c>
       <c r="F68" s="9" t="s">
-        <v>219</v>
+        <v>213</v>
       </c>
       <c r="G68" s="10" t="s">
-        <v>289</v>
+        <v>282</v>
       </c>
       <c r="H68" s="9" t="s">
-        <v>309</v>
+        <v>302</v>
       </c>
       <c r="I68" s="10" t="s">
-        <v>369</v>
+        <v>361</v>
       </c>
       <c r="J68" s="9">
         <v>2</v>
@@ -4005,25 +4024,25 @@
         <v>67</v>
       </c>
       <c r="C69" s="13" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D69" s="7" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="E69" s="8" t="s">
-        <v>171</v>
+        <v>167</v>
       </c>
       <c r="F69" s="7" t="s">
-        <v>216</v>
+        <v>210</v>
       </c>
       <c r="G69" s="8" t="s">
-        <v>290</v>
+        <v>283</v>
       </c>
       <c r="H69" s="7" t="s">
-        <v>309</v>
+        <v>302</v>
       </c>
       <c r="I69" s="8" t="s">
-        <v>370</v>
+        <v>362</v>
       </c>
       <c r="J69" s="7">
         <v>2</v>
@@ -4037,25 +4056,25 @@
         <v>68</v>
       </c>
       <c r="C70" s="13" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D70" s="9" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="E70" s="10" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="F70" s="9" t="s">
-        <v>217</v>
+        <v>211</v>
       </c>
       <c r="G70" s="10" t="s">
-        <v>291</v>
+        <v>284</v>
       </c>
       <c r="H70" s="9" t="s">
-        <v>309</v>
+        <v>302</v>
       </c>
       <c r="I70" s="10" t="s">
-        <v>371</v>
+        <v>363</v>
       </c>
       <c r="J70" s="9">
         <v>4</v>
@@ -4069,25 +4088,25 @@
         <v>69</v>
       </c>
       <c r="C71" s="12" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D71" s="7" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="E71" s="8" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="F71" s="7" t="s">
-        <v>216</v>
+        <v>210</v>
       </c>
       <c r="G71" s="8" t="s">
-        <v>292</v>
+        <v>285</v>
       </c>
       <c r="H71" s="7" t="s">
-        <v>309</v>
+        <v>302</v>
       </c>
       <c r="I71" s="8" t="s">
-        <v>372</v>
+        <v>364</v>
       </c>
       <c r="J71" s="7">
         <v>4</v>
@@ -4101,25 +4120,25 @@
         <v>70</v>
       </c>
       <c r="C72" s="13" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D72" s="9" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="E72" s="10" t="s">
-        <v>174</v>
+        <v>170</v>
       </c>
       <c r="F72" s="9" t="s">
-        <v>216</v>
+        <v>210</v>
       </c>
       <c r="G72" s="10" t="s">
-        <v>293</v>
+        <v>286</v>
       </c>
       <c r="H72" s="9" t="s">
-        <v>309</v>
+        <v>302</v>
       </c>
       <c r="I72" s="10" t="s">
-        <v>373</v>
+        <v>365</v>
       </c>
       <c r="J72" s="9">
         <v>8</v>
@@ -4133,25 +4152,25 @@
         <v>71</v>
       </c>
       <c r="C73" s="12" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D73" s="7" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="E73" s="8" t="s">
-        <v>175</v>
+        <v>171</v>
       </c>
       <c r="F73" s="7" t="s">
-        <v>216</v>
+        <v>210</v>
       </c>
       <c r="G73" s="8" t="s">
-        <v>294</v>
+        <v>287</v>
       </c>
       <c r="H73" s="7" t="s">
-        <v>309</v>
+        <v>302</v>
       </c>
       <c r="I73" s="8" t="s">
-        <v>363</v>
+        <v>355</v>
       </c>
       <c r="J73" s="7">
         <v>8</v>
@@ -4165,25 +4184,25 @@
         <v>72</v>
       </c>
       <c r="C74" s="13" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D74" s="9" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="E74" s="10" t="s">
-        <v>176</v>
+        <v>172</v>
       </c>
       <c r="F74" s="9" t="s">
-        <v>220</v>
+        <v>214</v>
       </c>
       <c r="G74" s="10" t="s">
-        <v>220</v>
+        <v>214</v>
       </c>
       <c r="H74" s="9" t="s">
-        <v>324</v>
+        <v>316</v>
       </c>
       <c r="I74" s="10" t="s">
-        <v>376</v>
+        <v>368</v>
       </c>
       <c r="J74" s="9">
         <v>2</v>
@@ -4197,13 +4216,13 @@
         <v>73</v>
       </c>
       <c r="C75" s="12" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D75" s="7" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="E75" s="8" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="F75" s="7">
         <v>760390015</v>
@@ -4212,10 +4231,10 @@
         <v>760390015</v>
       </c>
       <c r="H75" s="7" t="s">
-        <v>325</v>
+        <v>317</v>
       </c>
       <c r="I75" s="10" t="s">
-        <v>376</v>
+        <v>368</v>
       </c>
       <c r="J75" s="7">
         <v>1</v>
@@ -4229,25 +4248,25 @@
         <v>74</v>
       </c>
       <c r="C76" s="13" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D76" s="9" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="E76" s="10" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="F76" s="9" t="s">
-        <v>221</v>
+        <v>215</v>
       </c>
       <c r="G76" s="10" t="s">
-        <v>295</v>
+        <v>288</v>
       </c>
       <c r="H76" s="9" t="s">
-        <v>326</v>
+        <v>318</v>
       </c>
       <c r="I76" s="10" t="s">
-        <v>376</v>
+        <v>368</v>
       </c>
       <c r="J76" s="9">
         <v>1</v>
@@ -4261,25 +4280,25 @@
         <v>75</v>
       </c>
       <c r="C77" s="12" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D77" s="7" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="E77" s="8" t="s">
-        <v>179</v>
+        <v>175</v>
       </c>
       <c r="F77" s="7" t="s">
-        <v>222</v>
+        <v>216</v>
       </c>
       <c r="G77" s="8" t="s">
-        <v>296</v>
+        <v>289</v>
       </c>
       <c r="H77" s="7" t="s">
-        <v>322</v>
+        <v>314</v>
       </c>
       <c r="I77" s="10" t="s">
-        <v>376</v>
+        <v>368</v>
       </c>
       <c r="J77" s="7">
         <v>1</v>
@@ -4293,25 +4312,25 @@
         <v>76</v>
       </c>
       <c r="C78" s="13" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D78" s="9" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="E78" s="10" t="s">
-        <v>180</v>
+        <v>176</v>
       </c>
       <c r="F78" s="9" t="s">
-        <v>223</v>
+        <v>217</v>
       </c>
       <c r="G78" s="10" t="s">
-        <v>297</v>
+        <v>290</v>
       </c>
       <c r="H78" s="9" t="s">
-        <v>322</v>
+        <v>314</v>
       </c>
       <c r="I78" s="10" t="s">
-        <v>376</v>
+        <v>368</v>
       </c>
       <c r="J78" s="9">
         <v>1</v>
@@ -4325,25 +4344,25 @@
         <v>77</v>
       </c>
       <c r="C79" s="12" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D79" s="7" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="E79" s="8" t="s">
-        <v>181</v>
+        <v>177</v>
       </c>
       <c r="F79" s="7" t="s">
-        <v>224</v>
+        <v>218</v>
       </c>
       <c r="G79" s="8" t="s">
-        <v>298</v>
+        <v>291</v>
       </c>
       <c r="H79" s="7" t="s">
-        <v>322</v>
+        <v>314</v>
       </c>
       <c r="I79" s="10" t="s">
-        <v>376</v>
+        <v>368</v>
       </c>
       <c r="J79" s="7">
         <v>1</v>
@@ -4357,25 +4376,25 @@
         <v>78</v>
       </c>
       <c r="C80" s="13" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D80" s="9" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="E80" s="10" t="s">
-        <v>182</v>
+        <v>178</v>
       </c>
       <c r="F80" s="9" t="s">
-        <v>224</v>
+        <v>218</v>
       </c>
       <c r="G80" s="10" t="s">
-        <v>299</v>
+        <v>292</v>
       </c>
       <c r="H80" s="9" t="s">
-        <v>322</v>
+        <v>314</v>
       </c>
       <c r="I80" s="10" t="s">
-        <v>376</v>
+        <v>368</v>
       </c>
       <c r="J80" s="9">
         <v>1</v>
@@ -4389,25 +4408,25 @@
         <v>79</v>
       </c>
       <c r="C81" s="13" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D81" s="7" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="E81" s="8" t="s">
-        <v>183</v>
+        <v>179</v>
       </c>
       <c r="F81" s="7" t="s">
-        <v>225</v>
+        <v>219</v>
       </c>
       <c r="G81" s="8" t="s">
-        <v>300</v>
+        <v>293</v>
       </c>
       <c r="H81" s="7" t="s">
-        <v>327</v>
+        <v>319</v>
       </c>
       <c r="I81" s="10" t="s">
-        <v>376</v>
+        <v>368</v>
       </c>
       <c r="J81" s="7">
         <v>1</v>
@@ -4421,25 +4440,25 @@
         <v>80</v>
       </c>
       <c r="C82" s="13" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D82" s="9" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="E82" s="10" t="s">
-        <v>184</v>
+        <v>180</v>
       </c>
       <c r="F82" s="9" t="s">
-        <v>226</v>
+        <v>220</v>
       </c>
       <c r="G82" s="10" t="s">
-        <v>226</v>
+        <v>220</v>
       </c>
       <c r="H82" s="9" t="s">
-        <v>328</v>
+        <v>320</v>
       </c>
       <c r="I82" s="10" t="s">
-        <v>376</v>
+        <v>368</v>
       </c>
       <c r="J82" s="9">
         <v>1</v>
@@ -4456,22 +4475,22 @@
         <v>1</v>
       </c>
       <c r="D83" s="7" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="E83" s="8" t="s">
-        <v>185</v>
+        <v>181</v>
       </c>
       <c r="F83" s="7" t="s">
-        <v>227</v>
+        <v>221</v>
       </c>
       <c r="G83" s="8" t="s">
-        <v>227</v>
+        <v>221</v>
       </c>
       <c r="H83" s="7" t="s">
-        <v>329</v>
+        <v>321</v>
       </c>
       <c r="I83" s="10" t="s">
-        <v>376</v>
+        <v>368</v>
       </c>
       <c r="J83" s="7">
         <v>1</v>
@@ -4486,22 +4505,22 @@
       </c>
       <c r="C84" s="13"/>
       <c r="D84" s="9" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="E84" s="10" t="s">
-        <v>186</v>
+        <v>182</v>
       </c>
       <c r="F84" s="9" t="s">
-        <v>228</v>
+        <v>222</v>
       </c>
       <c r="G84" s="10" t="s">
-        <v>301</v>
+        <v>294</v>
       </c>
       <c r="H84" s="9" t="s">
-        <v>322</v>
+        <v>314</v>
       </c>
       <c r="I84" s="10" t="s">
-        <v>376</v>
+        <v>368</v>
       </c>
       <c r="J84" s="9">
         <v>1</v>
@@ -4515,25 +4534,25 @@
         <v>83</v>
       </c>
       <c r="C85" s="12" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D85" s="7" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="E85" s="8" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
       <c r="F85" s="7" t="s">
-        <v>229</v>
+        <v>223</v>
       </c>
       <c r="G85" s="8" t="s">
-        <v>302</v>
+        <v>295</v>
       </c>
       <c r="H85" s="7" t="s">
-        <v>322</v>
+        <v>314</v>
       </c>
       <c r="I85" s="10" t="s">
-        <v>376</v>
+        <v>368</v>
       </c>
       <c r="J85" s="7">
         <v>4</v>
@@ -4547,25 +4566,25 @@
         <v>84</v>
       </c>
       <c r="C86" s="13" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D86" s="9" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="E86" s="10" t="s">
-        <v>188</v>
+        <v>184</v>
       </c>
       <c r="F86" s="9" t="s">
-        <v>230</v>
+        <v>224</v>
       </c>
       <c r="G86" s="10" t="s">
-        <v>303</v>
+        <v>296</v>
       </c>
       <c r="H86" s="9" t="s">
-        <v>322</v>
+        <v>314</v>
       </c>
       <c r="I86" s="10" t="s">
-        <v>376</v>
+        <v>368</v>
       </c>
       <c r="J86" s="9">
         <v>2</v>
@@ -4579,25 +4598,25 @@
         <v>85</v>
       </c>
       <c r="C87" s="12" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D87" s="7" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="E87" s="8" t="s">
-        <v>189</v>
+        <v>185</v>
       </c>
       <c r="F87" s="7" t="s">
-        <v>231</v>
+        <v>225</v>
       </c>
       <c r="G87" s="8" t="s">
-        <v>304</v>
+        <v>297</v>
       </c>
       <c r="H87" s="7" t="s">
-        <v>322</v>
+        <v>314</v>
       </c>
       <c r="I87" s="10" t="s">
-        <v>376</v>
+        <v>368</v>
       </c>
       <c r="J87" s="7">
         <v>1</v>
@@ -4611,125 +4630,125 @@
         <v>86</v>
       </c>
       <c r="C88" s="13" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D88" s="9" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="E88" s="10" t="s">
-        <v>190</v>
+        <v>186</v>
       </c>
       <c r="F88" s="9" t="s">
-        <v>232</v>
+        <v>226</v>
       </c>
       <c r="G88" s="10" t="s">
-        <v>305</v>
+        <v>298</v>
       </c>
       <c r="H88" s="9" t="s">
-        <v>322</v>
+        <v>314</v>
       </c>
       <c r="I88" s="10" t="s">
-        <v>376</v>
+        <v>368</v>
       </c>
       <c r="J88" s="9">
         <v>8</v>
       </c>
       <c r="K88" s="9"/>
     </row>
-    <row r="89" spans="1:12" s="15" customFormat="1" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B89" s="16">
+    <row r="89" spans="1:12" s="14" customFormat="1" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B89" s="15">
         <f t="shared" ref="B89:B91" si="1">ROW(B89) - ROW($B$2)</f>
         <v>87</v>
       </c>
-      <c r="C89" s="17" t="s">
-        <v>375</v>
-      </c>
-      <c r="D89" s="18" t="s">
-        <v>376</v>
-      </c>
-      <c r="E89" s="18" t="s">
-        <v>377</v>
-      </c>
-      <c r="F89" s="18" t="s">
-        <v>376</v>
-      </c>
-      <c r="G89" s="19" t="s">
-        <v>378</v>
-      </c>
-      <c r="H89" s="18" t="s">
-        <v>379</v>
-      </c>
-      <c r="I89" s="19" t="s">
-        <v>376</v>
-      </c>
-      <c r="J89" s="18">
-        <v>1</v>
-      </c>
-      <c r="K89" s="18"/>
+      <c r="C89" s="16" t="s">
+        <v>367</v>
+      </c>
+      <c r="D89" s="17" t="s">
+        <v>368</v>
+      </c>
+      <c r="E89" s="17" t="s">
+        <v>369</v>
+      </c>
+      <c r="F89" s="17" t="s">
+        <v>368</v>
+      </c>
+      <c r="G89" s="18" t="s">
+        <v>370</v>
+      </c>
+      <c r="H89" s="17" t="s">
+        <v>371</v>
+      </c>
+      <c r="I89" s="18" t="s">
+        <v>368</v>
+      </c>
+      <c r="J89" s="17">
+        <v>1</v>
+      </c>
+      <c r="K89" s="17"/>
       <c r="L89"/>
     </row>
-    <row r="90" spans="1:12" s="15" customFormat="1" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B90" s="16">
+    <row r="90" spans="1:12" s="14" customFormat="1" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B90" s="15">
         <f t="shared" si="1"/>
         <v>88</v>
       </c>
-      <c r="C90" s="20" t="s">
-        <v>375</v>
-      </c>
-      <c r="D90" s="21" t="s">
+      <c r="C90" s="19" t="s">
+        <v>367</v>
+      </c>
+      <c r="D90" s="20" t="s">
+        <v>368</v>
+      </c>
+      <c r="E90" s="20" t="s">
         <v>376</v>
       </c>
-      <c r="E90" s="21" t="s">
-        <v>384</v>
-      </c>
-      <c r="F90" s="21" t="s">
-        <v>376</v>
-      </c>
-      <c r="G90" s="22" t="s">
-        <v>390</v>
-      </c>
-      <c r="H90" s="21" t="s">
-        <v>380</v>
-      </c>
-      <c r="I90" s="22" t="s">
-        <v>376</v>
-      </c>
-      <c r="J90" s="21">
-        <v>1</v>
-      </c>
-      <c r="K90" s="18"/>
+      <c r="F90" s="20" t="s">
+        <v>368</v>
+      </c>
+      <c r="G90" s="21" t="s">
+        <v>382</v>
+      </c>
+      <c r="H90" s="20" t="s">
+        <v>372</v>
+      </c>
+      <c r="I90" s="21" t="s">
+        <v>368</v>
+      </c>
+      <c r="J90" s="20">
+        <v>1</v>
+      </c>
+      <c r="K90" s="17"/>
       <c r="L90"/>
     </row>
-    <row r="91" spans="1:12" s="15" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B91" s="16">
+    <row r="91" spans="1:12" s="14" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B91" s="15">
         <f t="shared" si="1"/>
         <v>89</v>
       </c>
-      <c r="C91" s="23" t="s">
+      <c r="C91" s="22" t="s">
+        <v>367</v>
+      </c>
+      <c r="D91" s="23" t="s">
+        <v>368</v>
+      </c>
+      <c r="E91" s="23" t="s">
+        <v>373</v>
+      </c>
+      <c r="F91" s="23" t="s">
+        <v>368</v>
+      </c>
+      <c r="G91" s="24" t="s">
+        <v>374</v>
+      </c>
+      <c r="H91" s="23" t="s">
         <v>375</v>
       </c>
-      <c r="D91" s="24" t="s">
-        <v>376</v>
-      </c>
-      <c r="E91" s="24" t="s">
-        <v>381</v>
-      </c>
-      <c r="F91" s="24" t="s">
-        <v>376</v>
-      </c>
-      <c r="G91" s="25" t="s">
-        <v>382</v>
-      </c>
-      <c r="H91" s="24" t="s">
-        <v>383</v>
-      </c>
-      <c r="I91" s="25" t="s">
-        <v>376</v>
-      </c>
-      <c r="J91" s="24">
-        <v>1</v>
-      </c>
-      <c r="K91" s="26"/>
+      <c r="I91" s="24" t="s">
+        <v>368</v>
+      </c>
+      <c r="J91" s="23">
+        <v>1</v>
+      </c>
+      <c r="K91" s="25"/>
       <c r="L91"/>
     </row>
   </sheetData>

</xml_diff>